<commit_message>
Added graph tooltip validation and data extraction for dashboard charts
</commit_message>
<xml_diff>
--- a/downloads/consumers.xlsx
+++ b/downloads/consumers.xlsx
@@ -448,13 +448,13 @@
         <v>X2090346</v>
       </c>
       <c r="E2" t="str">
-        <v>9th Mar 2026 10:00:02 AM</v>
+        <v>11th Mar 2026 03:00:02 PM</v>
       </c>
       <c r="F2" t="str">
-        <v>0.000</v>
+        <v>NA</v>
       </c>
       <c r="G2" t="str">
-        <v>5700.000</v>
+        <v>NA</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -474,13 +474,13 @@
         <v>X1313762</v>
       </c>
       <c r="E3" t="str">
-        <v>9th Mar 2026 11:00:00 AM</v>
+        <v>11th Mar 2026 02:00:01 PM</v>
       </c>
       <c r="F3" t="str">
         <v>0.000</v>
       </c>
       <c r="G3" t="str">
-        <v>5280.000</v>
+        <v>8130.000</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -500,13 +500,13 @@
         <v>X1174645</v>
       </c>
       <c r="E4" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 02:00:01 PM</v>
       </c>
       <c r="F4" t="str">
         <v>0.000</v>
       </c>
       <c r="G4" t="str">
-        <v>50.000</v>
+        <v>60.000</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -526,13 +526,13 @@
         <v>X1972016</v>
       </c>
       <c r="E5" t="str">
-        <v>9th Mar 2026 11:00:02 AM</v>
+        <v>11th Mar 2026 02:00:00 PM</v>
       </c>
       <c r="F5" t="str">
         <v>0.000</v>
       </c>
       <c r="G5" t="str">
-        <v>330.000</v>
+        <v>1075.000</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -552,13 +552,13 @@
         <v>XE484946</v>
       </c>
       <c r="E6" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F6" t="str">
-        <v>0.000</v>
+        <v>NA</v>
       </c>
       <c r="G6" t="str">
-        <v>750.000</v>
+        <v>NA</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -604,13 +604,13 @@
         <v>XD471424</v>
       </c>
       <c r="E8" t="str">
-        <v>9th Mar 2026 11:00:00 AM</v>
+        <v>11th Mar 2026 03:00:00 PM</v>
       </c>
       <c r="F8" t="str">
-        <v>9900.000</v>
+        <v>NA</v>
       </c>
       <c r="G8" t="str">
-        <v>9900.000</v>
+        <v>NA</v>
       </c>
       <c r="H8">
         <v>7</v>
@@ -618,25 +618,25 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BI25GMRA0004</v>
+        <v>BI25GMRA0003</v>
       </c>
       <c r="B9" t="str">
-        <v>Multisorb Technologies</v>
+        <v>Cyient DLM</v>
       </c>
       <c r="C9" t="str">
-        <v>4100005439</v>
+        <v>4100006123</v>
       </c>
       <c r="D9" t="str">
-        <v>X2233641</v>
+        <v>X1244179</v>
       </c>
       <c r="E9" t="str">
-        <v>7th Mar 2026 02:15:00 PM</v>
+        <v>11th Mar 2026 02:00:01 PM</v>
       </c>
       <c r="F9" t="str">
-        <v>NA</v>
+        <v>0.000</v>
       </c>
       <c r="G9" t="str">
-        <v>NA</v>
+        <v>6560.000</v>
       </c>
       <c r="H9">
         <v>8</v>
@@ -656,13 +656,13 @@
         <v>23010551</v>
       </c>
       <c r="E10" t="str">
-        <v>9th Mar 2026 11:00:02 AM</v>
+        <v>11th Mar 2026 03:00:02 PM</v>
       </c>
       <c r="F10" t="str">
-        <v>400.000</v>
+        <v>NA</v>
       </c>
       <c r="G10" t="str">
-        <v>400.000</v>
+        <v>NA</v>
       </c>
       <c r="H10">
         <v>9</v>
@@ -682,7 +682,7 @@
         <v>X2090340</v>
       </c>
       <c r="E11" t="str">
-        <v>9th Mar 2026 11:45:01 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F11" t="str">
         <v>NA</v>
@@ -734,13 +734,13 @@
         <v>24021286</v>
       </c>
       <c r="E13" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F13" t="str">
-        <v>3530.000</v>
+        <v>NA</v>
       </c>
       <c r="G13" t="str">
-        <v>3530.000</v>
+        <v>NA</v>
       </c>
       <c r="H13">
         <v>12</v>
@@ -748,25 +748,25 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BI25GMRA0003</v>
+        <v>BI25GMRA0004</v>
       </c>
       <c r="B14" t="str">
-        <v>Cyient DLM</v>
+        <v>Multisorb Technologies</v>
       </c>
       <c r="C14" t="str">
-        <v>4100006123</v>
+        <v>4100005439</v>
       </c>
       <c r="D14" t="str">
-        <v>X1244179</v>
+        <v>X2233641</v>
       </c>
       <c r="E14" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>7th Mar 2026 02:15:00 PM</v>
       </c>
       <c r="F14" t="str">
-        <v>0.000</v>
+        <v>NA</v>
       </c>
       <c r="G14" t="str">
-        <v>480.000</v>
+        <v>NA</v>
       </c>
       <c r="H14">
         <v>13</v>
@@ -786,13 +786,13 @@
         <v>X2091454</v>
       </c>
       <c r="E15" t="str">
-        <v>9th Mar 2026 11:00:02 AM</v>
+        <v>11th Mar 2026 02:00:01 PM</v>
       </c>
       <c r="F15" t="str">
         <v>0.000</v>
       </c>
       <c r="G15" t="str">
-        <v>165.000</v>
+        <v>330.000</v>
       </c>
       <c r="H15">
         <v>14</v>
@@ -812,13 +812,13 @@
         <v>23010587</v>
       </c>
       <c r="E16" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 02:00:02 PM</v>
       </c>
       <c r="F16" t="str">
-        <v>6100.000</v>
+        <v>8500.000</v>
       </c>
       <c r="G16" t="str">
-        <v>6100.000</v>
+        <v>8500.000</v>
       </c>
       <c r="H16">
         <v>15</v>
@@ -826,25 +826,25 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>BI25GMRA0001</v>
+        <v>BI25GMRA0002</v>
       </c>
       <c r="B17" t="str">
-        <v>GMR AERO TOWER 2 INCOMER</v>
+        <v>Cronus Pharma</v>
       </c>
       <c r="C17" t="str">
-        <v>CON-1002</v>
+        <v>4100005169</v>
       </c>
       <c r="D17" t="str">
-        <v>18132429</v>
+        <v>X1580068</v>
       </c>
       <c r="E17" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>10th Mar 2026 04:00:02 PM</v>
       </c>
       <c r="F17" t="str">
-        <v>3800.000</v>
+        <v>NA</v>
       </c>
       <c r="G17" t="str">
-        <v>3800.000</v>
+        <v>NA</v>
       </c>
       <c r="H17">
         <v>16</v>
@@ -852,25 +852,25 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>BI25GMRA0002</v>
+        <v>BI25GMRA0001</v>
       </c>
       <c r="B18" t="str">
-        <v>Cronus Pharma</v>
+        <v>GMR AERO TOWER 2 INCOMER</v>
       </c>
       <c r="C18" t="str">
-        <v>4100005169</v>
+        <v>CON-1002</v>
       </c>
       <c r="D18" t="str">
-        <v>X1580068</v>
+        <v>18132429</v>
       </c>
       <c r="E18" t="str">
-        <v>9th Mar 2026 11:00:00 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F18" t="str">
-        <v>0.000</v>
+        <v>NA</v>
       </c>
       <c r="G18" t="str">
-        <v>22380.000</v>
+        <v>NA</v>
       </c>
       <c r="H18">
         <v>17</v>
@@ -890,13 +890,13 @@
         <v>X2199608</v>
       </c>
       <c r="E19" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F19" t="str">
-        <v>2460.000</v>
+        <v>NA</v>
       </c>
       <c r="G19" t="str">
-        <v>2460.000</v>
+        <v>NA</v>
       </c>
       <c r="H19">
         <v>18</v>
@@ -916,13 +916,13 @@
         <v>24021328</v>
       </c>
       <c r="E20" t="str">
-        <v>9th Mar 2026 11:00:01 AM</v>
+        <v>11th Mar 2026 03:00:01 PM</v>
       </c>
       <c r="F20" t="str">
-        <v>820.000</v>
+        <v>NA</v>
       </c>
       <c r="G20" t="str">
-        <v>820.000</v>
+        <v>NA</v>
       </c>
       <c r="H20">
         <v>19</v>

</xml_diff>

<commit_message>
Added failure email notification and Allure report deployment
</commit_message>
<xml_diff>
--- a/downloads/consumers.xlsx
+++ b/downloads/consumers.xlsx
@@ -448,13 +448,13 @@
         <v>X2090346</v>
       </c>
       <c r="E2" t="str">
-        <v>11th Mar 2026 03:00:02 PM</v>
+        <v>13th Mar 2026 12:00:00 PM</v>
       </c>
       <c r="F2" t="str">
-        <v>NA</v>
+        <v>0.000</v>
       </c>
       <c r="G2" t="str">
-        <v>NA</v>
+        <v>6670.000</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -474,13 +474,13 @@
         <v>X1313762</v>
       </c>
       <c r="E3" t="str">
-        <v>11th Mar 2026 02:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F3" t="str">
         <v>0.000</v>
       </c>
       <c r="G3" t="str">
-        <v>8130.000</v>
+        <v>6890.000</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -500,13 +500,13 @@
         <v>X1174645</v>
       </c>
       <c r="E4" t="str">
-        <v>11th Mar 2026 02:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F4" t="str">
         <v>0.000</v>
       </c>
       <c r="G4" t="str">
-        <v>60.000</v>
+        <v>55.000</v>
       </c>
       <c r="H4">
         <v>3</v>
@@ -526,13 +526,13 @@
         <v>X1972016</v>
       </c>
       <c r="E5" t="str">
-        <v>11th Mar 2026 02:00:00 PM</v>
+        <v>13th Mar 2026 12:00:02 PM</v>
       </c>
       <c r="F5" t="str">
         <v>0.000</v>
       </c>
       <c r="G5" t="str">
-        <v>1075.000</v>
+        <v>1115.000</v>
       </c>
       <c r="H5">
         <v>4</v>
@@ -552,13 +552,13 @@
         <v>XE484946</v>
       </c>
       <c r="E6" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F6" t="str">
-        <v>NA</v>
+        <v>0.000</v>
       </c>
       <c r="G6" t="str">
-        <v>NA</v>
+        <v>2700.000</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -604,7 +604,7 @@
         <v>XD471424</v>
       </c>
       <c r="E8" t="str">
-        <v>11th Mar 2026 03:00:00 PM</v>
+        <v>12th Mar 2026 11:00:01 AM</v>
       </c>
       <c r="F8" t="str">
         <v>NA</v>
@@ -630,13 +630,13 @@
         <v>X1244179</v>
       </c>
       <c r="E9" t="str">
-        <v>11th Mar 2026 02:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F9" t="str">
         <v>0.000</v>
       </c>
       <c r="G9" t="str">
-        <v>6560.000</v>
+        <v>6020.000</v>
       </c>
       <c r="H9">
         <v>8</v>
@@ -656,13 +656,13 @@
         <v>23010551</v>
       </c>
       <c r="E10" t="str">
-        <v>11th Mar 2026 03:00:02 PM</v>
+        <v>13th Mar 2026 12:00:00 PM</v>
       </c>
       <c r="F10" t="str">
-        <v>NA</v>
+        <v>1100.000</v>
       </c>
       <c r="G10" t="str">
-        <v>NA</v>
+        <v>1100.000</v>
       </c>
       <c r="H10">
         <v>9</v>
@@ -682,13 +682,13 @@
         <v>X2090340</v>
       </c>
       <c r="E11" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:15:01 PM</v>
       </c>
       <c r="F11" t="str">
-        <v>NA</v>
+        <v>0.000</v>
       </c>
       <c r="G11" t="str">
-        <v>NA</v>
+        <v>6040.000</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -734,13 +734,13 @@
         <v>24021286</v>
       </c>
       <c r="E13" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F13" t="str">
-        <v>NA</v>
+        <v>14070.000</v>
       </c>
       <c r="G13" t="str">
-        <v>NA</v>
+        <v>14080.000</v>
       </c>
       <c r="H13">
         <v>12</v>
@@ -786,13 +786,13 @@
         <v>X2091454</v>
       </c>
       <c r="E15" t="str">
-        <v>11th Mar 2026 02:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F15" t="str">
         <v>0.000</v>
       </c>
       <c r="G15" t="str">
-        <v>330.000</v>
+        <v>335.000</v>
       </c>
       <c r="H15">
         <v>14</v>
@@ -812,13 +812,13 @@
         <v>23010587</v>
       </c>
       <c r="E16" t="str">
-        <v>11th Mar 2026 02:00:02 PM</v>
+        <v>13th Mar 2026 12:00:02 PM</v>
       </c>
       <c r="F16" t="str">
-        <v>8500.000</v>
+        <v>9000.000</v>
       </c>
       <c r="G16" t="str">
-        <v>8500.000</v>
+        <v>9100.000</v>
       </c>
       <c r="H16">
         <v>15</v>
@@ -838,13 +838,13 @@
         <v>X1580068</v>
       </c>
       <c r="E17" t="str">
-        <v>10th Mar 2026 04:00:02 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F17" t="str">
-        <v>NA</v>
+        <v>0.000</v>
       </c>
       <c r="G17" t="str">
-        <v>NA</v>
+        <v>23310.000</v>
       </c>
       <c r="H17">
         <v>16</v>
@@ -864,13 +864,13 @@
         <v>18132429</v>
       </c>
       <c r="E18" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:01:30 PM</v>
       </c>
       <c r="F18" t="str">
-        <v>NA</v>
+        <v>7100.000</v>
       </c>
       <c r="G18" t="str">
-        <v>NA</v>
+        <v>7100.000</v>
       </c>
       <c r="H18">
         <v>17</v>
@@ -890,13 +890,13 @@
         <v>X2199608</v>
       </c>
       <c r="E19" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F19" t="str">
-        <v>NA</v>
+        <v>3360.000</v>
       </c>
       <c r="G19" t="str">
-        <v>NA</v>
+        <v>3380.000</v>
       </c>
       <c r="H19">
         <v>18</v>
@@ -916,13 +916,13 @@
         <v>24021328</v>
       </c>
       <c r="E20" t="str">
-        <v>11th Mar 2026 03:00:01 PM</v>
+        <v>13th Mar 2026 12:00:01 PM</v>
       </c>
       <c r="F20" t="str">
-        <v>NA</v>
+        <v>360.000</v>
       </c>
       <c r="G20" t="str">
-        <v>NA</v>
+        <v>360.000</v>
       </c>
       <c r="H20">
         <v>19</v>

</xml_diff>